<commit_message>
Restore D6 v1.2 scoring contract
</commit_message>
<xml_diff>
--- a/Project 1 Data Quality Assessment/D6 Parallel-redundancy Temporal Consistency/outputs/data/D6_audit_log.xlsx
+++ b/Project 1 Data Quality Assessment/D6 Parallel-redundancy Temporal Consistency/outputs/data/D6_audit_log.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,7 +454,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>D6V13_20260713_103039</t>
+          <t>D6V14_20260714_024929</t>
         </is>
       </c>
     </row>
@@ -466,105 +466,141 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>d6-v1.3-independent-20260713</t>
+          <t>d6-v1.4-restored-v12-20260714</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>generated_utc</t>
+          <t>calibration_id</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-13T10:34:45.441000+00:00</t>
+          <t>D6CAL-V14-20f697901061</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>d2_run_id</t>
+          <t>generated_utc</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>D2V1_20260710_1733</t>
+          <t>2026-07-14T02:51:51.905879+00:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>d2_calibration_id</t>
+          <t>d2_run_id</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>NorthBank_D2_v1_20260710</t>
+          <t>D2V1_20260710_1733</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>n_rows</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>42847</v>
+          <t>d2_calibration_id</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>NorthBank_D2_v1_20260710</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>n_pairs</t>
+          <t>n_rows</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>7</v>
+        <v>42847</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>data_start</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="n">
-        <v>45870</v>
+          <t>n_pairs</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>data_end</t>
+          <t>data_start</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>46125.99305555555</v>
+        <v>45870</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>evaluable_rate</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>0.7909771979368451</v>
+          <t>data_end</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>46125.99305555555</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>evaluable_rate_D6_raw</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.7909771979368451</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>D6_forDQR_status</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>provisional only; pending D7 arbitration</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>benchmark_D7_screen</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>pending; no D7 proxy generated</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>causal_claim</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>pair asymmetry only; sensor/process cause unresolved</t>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>pair asymmetry only; sensor/process cause pending D7</t>
         </is>
       </c>
     </row>
@@ -579,7 +615,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -673,22 +709,110 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>regime_templates</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>D1_regime_templates.xlsx</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>cf4bd67afd8248d8b8bf0a92a549bb1c28504f1fea4e7cf2b443b7e6b0123153</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2026-07-10T02:49:40.805057+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
           <t>d2_scores</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>D2_main_scores_hourly.xlsx</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>3f233f4add980824db243db71fc0c0a9844742239c378bb5ca20d97a48720df0</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>2026-07-10T09:35:03.368662+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>d6_config</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>d6.yaml</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1f0305e3d5a3eba54d7b3118975e967150b40f2789d22854210c7689533804dc</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2026-07-14T02:20:41.598806+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>d6_pipeline_code</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>pipeline.py</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>7b292b9f43248597dd9ac5974a343ae511f06bcbab8b5f5151fc1c9e96f7b927</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2026-07-14T02:48:27.198285+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>d6_scoring_code</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>scoring.py</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>9ff54d52d996449efd7630afdfa99bc9d2969e2e796e976d4932e998e99b0f76</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2026-07-14T02:37:11.533384+00:00</t>
         </is>
       </c>
     </row>
@@ -709,7 +833,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>rule</t>
+          <t>layer</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -719,7 +843,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>score_changed</t>
+          <t>output</t>
         </is>
       </c>
     </row>
@@ -731,41 +855,47 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>evaluation gate only</t>
-        </is>
-      </c>
-      <c r="C2" t="b">
-        <v>0</v>
+          <t>gate D6 evaluability</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>usable_for_D6</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>D1 sensor health</t>
+          <t>D1 bilateral fuse</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>interpretation context only</t>
-        </is>
-      </c>
-      <c r="C3" t="b">
-        <v>0</v>
+          <t>true v1.2 fuse</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>D6_after_D1</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>D7 spatial consensus</t>
+          <t>D7 zone consensus</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>not available; reserved for DQR evidence fusion</t>
-        </is>
-      </c>
-      <c r="C4" t="b">
-        <v>0</v>
+          <t>not available; no proxy generated</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>pending_D7_arbitration</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Release D1 and refresh dependent quality modules
</commit_message>
<xml_diff>
--- a/Project 1 Data Quality Assessment/D6 Parallel-redundancy Temporal Consistency/outputs/data/D6_audit_log.xlsx
+++ b/Project 1 Data Quality Assessment/D6 Parallel-redundancy Temporal Consistency/outputs/data/D6_audit_log.xlsx
@@ -454,7 +454,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>D6V14_20260714_024929</t>
+          <t>D6V14_20260722_021007</t>
         </is>
       </c>
     </row>
@@ -478,7 +478,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>D6CAL-V14-20f697901061</t>
+          <t>D6CAL-V14-d21144ef1b41</t>
         </is>
       </c>
     </row>
@@ -490,7 +490,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-14T02:51:51.905879+00:00</t>
+          <t>2026-07-22T02:12:16.734209+00:00</t>
         </is>
       </c>
     </row>
@@ -697,12 +697,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>abb941ac70ae2a0b94e081a6573cee472ea7681a93fb4d5a9b8113dcec8bd7e3</t>
+          <t>c825b4481c54a81f2d75d486183afd3ddea01593965b9bdef97d4277b44bbf78</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-07-10T02:49:31.813900+00:00</t>
+          <t>2026-07-22T02:04:23.222556+00:00</t>
         </is>
       </c>
     </row>
@@ -719,12 +719,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>cf4bd67afd8248d8b8bf0a92a549bb1c28504f1fea4e7cf2b443b7e6b0123153</t>
+          <t>7dba5c980a567645fff62ba3b46369ce2187498ee2e45e5abf4f25b0c6052d53</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-07-10T02:49:40.805057+00:00</t>
+          <t>2026-07-22T02:04:32.507595+00:00</t>
         </is>
       </c>
     </row>
@@ -785,12 +785,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>7b292b9f43248597dd9ac5974a343ae511f06bcbab8b5f5151fc1c9e96f7b927</t>
+          <t>c2243a6990ed1831fbed1694d6cd08b1e0d10a7efcb43d76cd47fd8ef43ecc48</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-07-14T02:48:27.198285+00:00</t>
+          <t>2026-07-22T02:04:05.834526+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>